<commit_message>
Eliminados bloques visuales cuadrados de los botones de navegacion en la cabecera del calendario modal (iconos circulares limpios)
</commit_message>
<xml_diff>
--- a/data/Reporte_Ventas_Inego_Consolidado.xlsx
+++ b/data/Reporte_Ventas_Inego_Consolidado.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -526,7 +526,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Desde: Inicio | Hasta: Actualidad | Generado: 2026-09-03 08:33</t>
+          <t>Desde: Inicio | Hasta: Actualidad | Generado: 2026-09-03 10:39</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Facturada</t>
         </is>
       </c>
       <c r="G6" s="9" t="n">
@@ -652,17 +652,17 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>COT-20260828-084029</t>
+          <t>COT-20260827-102419</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>jorge</t>
+          <t>Sebastián Guillermo Menoscal</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -681,36 +681,36 @@
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>10000</v>
+        <v>149.5</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>11500</v>
+        <v>171.925</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>COT-20260828-101827</t>
+          <t>COT-20260826-213811</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>jorge</t>
+          <t>Carlos Max Campoverde</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>B2C</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>0 (Contado)</t>
+          <t>72 días</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -719,36 +719,36 @@
         </is>
       </c>
       <c r="G8" s="9" t="n">
-        <v>12675</v>
+        <v>337.25</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>14576.25</v>
+        <v>387.8375</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>COT-20260828-101851</t>
+          <t>COT-20260825-212633</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>jorge</t>
+          <t>Cliente de Prueba B2B S.A.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>B2C</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>0 (Contado)</t>
+          <t>72 días</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -757,36 +757,36 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>12000</v>
+        <v>75</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>13800</v>
+        <v>86.25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>COT-20260827-102419</t>
+          <t>COT-20260819-175711</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Sebastián Guillermo Menoscal</t>
+          <t>Cliente de Prueba B2B S.A.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>B2C</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>0 (Contado)</t>
+          <t>72 días</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -795,36 +795,36 @@
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>149.5</v>
+        <v>75</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>171.925</v>
+        <v>86.25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>COT-20260827-105647</t>
+          <t>COT-20260819-181108</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>jorge</t>
+          <t>Cliente de Prueba B2B S.A.</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>B2C</t>
+          <t>B2B</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>0 (Contado)</t>
+          <t>72 días</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -833,26 +833,26 @@
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>46150</v>
+        <v>75</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>53072.5</v>
+        <v>86.25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>COT-20260826-213811</t>
+          <t>COT-2026-001</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Carlos Max Campoverde</t>
+          <t>Ministerio de Obras Públicas Zonal 8</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -871,210 +871,58 @@
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>337.25</v>
+        <v>1500</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>387.8375</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>COT-20260825-212633</t>
+          <t>COT-2026-002</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Cliente de Prueba B2B S.A.</t>
+          <t>Juan Fernando Gómez</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>B2B</t>
+          <t>B2C</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>72 días</t>
+          <t>0 (Contado)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Facturada</t>
+          <t>Aprobada</t>
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>86.25</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>COT-20260819-175711</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Cliente de Prueba B2B S.A.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>72 días</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Facturada</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>75</v>
-      </c>
-      <c r="H14" s="9" t="n">
-        <v>86.25</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>COT-20260819-181108</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Cliente de Prueba B2B S.A.</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>72 días</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Facturada</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>75</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>86.25</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>COT-2026-001</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Ministerio de Obras Públicas Zonal 8</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>72 días</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Facturada</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>1725</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>COT-2026-002</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Juan Fernando Gómez</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>B2C</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>0 (Contado)</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Aprobada</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>120</v>
-      </c>
-      <c r="H17" s="6" t="n">
         <v>138</v>
       </c>
     </row>
-    <row r="18" ht="25" customHeight="1">
-      <c r="F18" s="10" t="inlineStr">
+    <row r="14" ht="25" customHeight="1">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>TOTAL GENERAL:</t>
         </is>
       </c>
-      <c r="H18" s="11" t="n">
-        <v>96453.66250000001</v>
+      <c r="H14" s="11" t="n">
+        <v>3504.9125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trasladada la tarjeta de 'Cálculo de Bono Mensual - Ingreso Manual' al módulo de Nómina y Roles de Pago de Socios (PayrollView.qml)
</commit_message>
<xml_diff>
--- a/data/Reporte_Ventas_Inego_Consolidado.xlsx
+++ b/data/Reporte_Ventas_Inego_Consolidado.xlsx
@@ -526,7 +526,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Desde: Inicio | Hasta: Actualidad | Generado: 2026-09-03 10:39</t>
+          <t>Desde: Inicio | Hasta: Actualidad | Generado: 2026-09-03 10:52</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Facturada</t>
         </is>
       </c>
       <c r="G5" s="6" t="n">

</xml_diff>

<commit_message>
feat: Sincronizacion total de modificaciones de cotizaciones, nomina de socios y optimizaciones de rendimiento
</commit_message>
<xml_diff>
--- a/data/Reporte_Ventas_Inego_Consolidado.xlsx
+++ b/data/Reporte_Ventas_Inego_Consolidado.xlsx
@@ -47,11 +47,13 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00C2410C"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -113,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -122,22 +124,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -503,17 +516,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="66" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="101" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -526,7 +550,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Desde: Inicio | Hasta: Actualidad | Generado: 2026-09-03 10:52</t>
+          <t>Desde: Inicio | Hasta: Actualidad | Generado: 2026-09-04 10:54</t>
         </is>
       </c>
     </row>
@@ -544,36 +568,91 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Cliente / Razón Social</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>RUC / Cédula</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>Tipo Cliente</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Días Crédito</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Subtotal ($)</t>
-        </is>
-      </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Total USD ($)</t>
+          <t>Aplica Retención SRI</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Producto / Ítem (Lista Desglosada)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Cant.</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>P. Unit ($)</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Subtotal Ítem ($)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Subtotal Trans. ($)</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>IVA 15% ($)</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Total Facturado ($)</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Ret. IR 1.75% ($)</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Ret. IVA 30% ($)</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Total Retenciones ($)</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>Valor Neto a Cobrar ($)</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>COT-20260903-083238</t>
@@ -591,342 +670,884 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
+          <t>0930860044</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>72 días</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>No (Cédula 10 dígitos / Consumidor Final)</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>• Licencia Microsoft Office 365 Professional (SOFT-001)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="M5" s="7" t="n">
         <v>272</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="N5" s="7" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="O5" s="7" t="n">
         <v>312.8</v>
       </c>
+      <c r="P5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="8" t="n">
+        <v>312.8</v>
+      </c>
     </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>COT-20260903-083303</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>COT-20260827-102419</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Sebastián Guillermo Menoscal</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>0920000072</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>0 (Contado)</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G6" s="9" t="n">
-        <v>444</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>510.6</v>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>No (Cédula 10 dígitos / Consumidor Final)</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>• Taladro Perforador 800W (FER-555)</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>149.5</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>22.425</v>
+      </c>
+      <c r="O6" s="12" t="n">
+        <v>171.93</v>
+      </c>
+      <c r="P6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="13" t="n">
+        <v>171.93</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>COT-20260827-102419</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Sebastián Guillermo Menoscal</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>0920000072</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>0 (Contado)</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>No (Cédula 10 dígitos / Consumidor Final)</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>• Producto de Prueba (PRD-TEST)</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="M7" s="12" t="n">
         <v>149.5</v>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>171.925</v>
+      <c r="N7" s="12" t="n">
+        <v>22.425</v>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>171.93</v>
+      </c>
+      <c r="P7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="13" t="n">
+        <v>171.93</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>COT-20260826-213811</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Carlos Max Campoverde</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>0930860044</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>72 días</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>No (Cédula 10 dígitos / Consumidor Final)</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>• Licencia Microsoft Office 365 Professional (SOFT-001)</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>169</v>
+      </c>
+      <c r="M8" s="7" t="n">
         <v>337.25</v>
       </c>
-      <c r="H8" s="9" t="n">
-        <v>387.8375</v>
+      <c r="N8" s="7" t="n">
+        <v>50.5875</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>387.84</v>
+      </c>
+      <c r="P8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="8" t="n">
+        <v>387.84</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>COT-20260826-213811</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Carlos Max Campoverde</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>0930860044</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>72 días</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Facturada</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>No (Cédula 10 dígitos / Consumidor Final)</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>• Tornillo Hexagonal 3/8 (PRD-004)</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>1.5625</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>337.25</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>50.5875</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>387.84</v>
+      </c>
+      <c r="P9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="8" t="n">
+        <v>387.84</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>COT-20260826-213811</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Carlos Max Campoverde</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>0930860044</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>72 días</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Facturada</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>No (Cédula 10 dígitos / Consumidor Final)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>• Licencia Microsoft Office 365 Professional - Proveedor: Importadora Central Quito (SOFT-001-LNK)</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>74.75</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>149.5</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>337.25</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>50.5875</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>387.84</v>
+      </c>
+      <c r="P10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="8" t="n">
+        <v>387.84</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
           <t>COT-20260825-212633</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Cliente de Prueba B2B S.A.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>0920000064001</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>72 días</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Sí (RUC 1.75% IR | 30% IVA)</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>• Ítem Comercial General (PROD-GEN)</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>75</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="L11" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="O11" s="12" t="n">
         <v>86.25</v>
       </c>
+      <c r="P11" s="12" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="Q11" s="12" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="R11" s="14" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="S11" s="13" t="n">
+        <v>81.56</v>
+      </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>COT-20260819-175711</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Cliente de Prueba B2B S.A.</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>0920000023001</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>72 días</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Sí (RUC 1.75% IR | 30% IVA)</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>• Ítem Comercial General (PROD-GEN)</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="7" t="n">
         <v>75</v>
       </c>
-      <c r="H10" s="9" t="n">
+      <c r="L12" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="O12" s="7" t="n">
         <v>86.25</v>
       </c>
+      <c r="P12" s="7" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="Q12" s="7" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="R12" s="15" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>81.56</v>
+      </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>COT-20260819-181108</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>Cliente de Prueba B2B S.A.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>0920000031001</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>72 días</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Sí (RUC 1.75% IR | 30% IVA)</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>• Ítem Comercial General (PROD-GEN)</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="12" t="n">
         <v>75</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="L13" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="N13" s="12" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="O13" s="12" t="n">
         <v>86.25</v>
       </c>
+      <c r="P13" s="12" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="Q13" s="12" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="R13" s="14" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="S13" s="13" t="n">
+        <v>81.56</v>
+      </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>COT-2026-001</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Ministerio de Obras Públicas Zonal 8</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>0960001110001</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>72 días</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Facturada</t>
         </is>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Sí (RUC 1.75% IR | 30% IVA)</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>• Ítem Comercial General (PROD-GEN)</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="L14" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>225</v>
+      </c>
+      <c r="O14" s="7" t="n">
         <v>1725</v>
       </c>
+      <c r="P14" s="7" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="Q14" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R14" s="15" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="S14" s="8" t="n">
+        <v>1631.25</v>
+      </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>COT-2026-002</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Juan Fernando Gómez</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>0920000015</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>B2C</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>0 (Contado)</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>Aprobada</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>No (Cédula 10 dígitos / Consumidor Final)</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>• Licencia Microsoft Office 365 Professional (SOFT-001)</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>65</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="M15" s="12" t="n">
         <v>120</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="N15" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="O15" s="12" t="n">
         <v>138</v>
       </c>
+      <c r="P15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="13" t="n">
+        <v>138</v>
+      </c>
     </row>
-    <row r="14" ht="25" customHeight="1">
-      <c r="F14" s="10" t="inlineStr">
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>TOTAL GENERAL:</t>
         </is>
       </c>
-      <c r="H14" s="11" t="n">
-        <v>3504.9125</v>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n"/>
+      <c r="J16" s="17" t="n"/>
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="17" t="n"/>
+      <c r="M16" s="18">
+        <f>SUM(M5:M15)</f>
+        <v/>
+      </c>
+      <c r="N16" s="18">
+        <f>SUM(N5:N15)</f>
+        <v/>
+      </c>
+      <c r="O16" s="18">
+        <f>SUM(O5:O15)</f>
+        <v/>
+      </c>
+      <c r="P16" s="18">
+        <f>SUM(P5:P15)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="18">
+        <f>SUM(Q5:Q15)</f>
+        <v/>
+      </c>
+      <c r="R16" s="18">
+        <f>SUM(R5:R15)</f>
+        <v/>
+      </c>
+      <c r="S16" s="18">
+        <f>SUM(S5:S15)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A16:L16"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>